<commit_message>
melhoria7 - melhoria planilha financeira
</commit_message>
<xml_diff>
--- a/public/Planilha-modelo.xlsx
+++ b/public/Planilha-modelo.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard Financeiro" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Controle" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,72 +20,81 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
-  <si>
-    <t xml:space="preserve">CONTROLE DE FINANÇAS PESSOAIS</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+  <si>
+    <t xml:space="preserve">CONTROLE DE FINANÇAS</t>
   </si>
   <si>
     <t xml:space="preserve">RECEITA TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">DESPESA TOTAL</t>
+    <t xml:space="preserve">Despesa TOTAL</t>
   </si>
   <si>
     <t xml:space="preserve">SALDO ATUAL</t>
   </si>
   <si>
-    <t xml:space="preserve">R$ 2,500.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$ 490.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$ 2,010.00</t>
-  </si>
-  <si>
     <t xml:space="preserve">DATA</t>
   </si>
   <si>
-    <t xml:space="preserve">TIPO</t>
+    <t xml:space="preserve">DESCRIÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CATEGORIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
   </si>
   <si>
     <t xml:space="preserve">VALOR</t>
   </si>
   <si>
-    <t xml:space="preserve">CATEGORIA</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-01-05</t>
   </si>
   <si>
+    <t xml:space="preserve">Recebimento Salário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salário</t>
+  </si>
+  <si>
     <t xml:space="preserve">Receita</t>
   </si>
   <si>
-    <t xml:space="preserve">Salário</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-01-07</t>
   </si>
   <si>
+    <t xml:space="preserve">Supermercado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimentação</t>
+  </si>
+  <si>
     <t xml:space="preserve">Despesa</t>
   </si>
   <si>
-    <t xml:space="preserve">Alimentação</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-01-15</t>
   </si>
   <si>
+    <t xml:space="preserve">Combustível</t>
+  </si>
+  <si>
     <t xml:space="preserve">Transporte</t>
   </si>
   <si>
     <t xml:space="preserve">2026-01-20</t>
   </si>
   <si>
+    <t xml:space="preserve">Cinema</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lazer</t>
   </si>
   <si>
     <t xml:space="preserve">2026-01-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projeto Freelance</t>
   </si>
   <si>
     <t xml:space="preserve">Freelance</t>
@@ -95,11 +104,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="&quot;R$ &quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$R$-416]\ #,##0.00;[RED]\-[$R$-416]\ #,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,66 +133,56 @@
       <family val="0"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="22"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF2E7D32"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FFC9211E"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="18"/>
       <color rgb="FF1A237E"/>
-      <name val="Segoe UI Semibold"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF757575"/>
-      <name val="Segoe UI"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FF2E7D32"/>
-      <name val="Segoe UI Bold"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FFC62828"/>
-      <name val="Segoe UI Bold"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF1A237E"/>
-      <name val="Segoe UI Bold"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Segoe UI Bold"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF212121"/>
-      <name val="Segoe UI"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF2E7D32"/>
-      <name val="Segoe UI Bold"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFC62828"/>
-      <name val="Segoe UI Bold"/>
+      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -196,14 +196,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5F5F5"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FF1A237E"/>
+        <bgColor rgb="FF333399"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A237E"/>
-        <bgColor rgb="FF333399"/>
+        <fgColor rgb="FFF9F9F9"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -217,16 +217,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FFBDBDBD"/>
+        <color rgb="FFDDDDDD"/>
       </left>
       <right style="thin">
-        <color rgb="FFBDBDBD"/>
+        <color rgb="FFDDDDDD"/>
       </right>
       <top style="thin">
-        <color rgb="FFBDBDBD"/>
+        <color rgb="FFDDDDDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFBDBDBD"/>
+        <color rgb="FFDDDDDD"/>
       </bottom>
       <diagonal/>
     </border>
@@ -256,69 +256,57 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -346,16 +334,16 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFBDBDBD"/>
-      <rgbColor rgb="FF757575"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF5F5F5"/>
+      <rgbColor rgb="FFF9F9F9"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FFDDDDDD"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -384,10 +372,10 @@
       <rgbColor rgb="FF2E7D32"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FFC62828"/>
+      <rgbColor rgb="FFC9211E"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF212121"/>
+      <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -573,221 +561,170 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:E27"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:F14"/>
+  <sheetFormatPr defaultColWidth="20.4609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.46"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3" t="s">
+    <row r="6" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="n">
+        <f aca="false">SUMIF(E10:E500,"Receita",F10:F500)</f>
+        <v>2500</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <f aca="false">SUMIF(E10:E500,"Despesa",F10:F500)</f>
+        <v>490</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <f aca="false">B6-D6</f>
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D9" s="8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="6" t="s">
+      <c r="E9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="F9" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="6" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="C10" s="9" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="7" t="s">
+      <c r="D10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="F10" s="10" t="n">
         <v>2000</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>300</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="13" t="n">
+      <c r="E12" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="E11" s="14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="8" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="F14" s="10" t="n">
         <v>500</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="7"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="7"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="7"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="7"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="7"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="7"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="10"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="7"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="7"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="10"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="7"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="10"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="7"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="10"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="7"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="7"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="10"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="7"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="10"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="7"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="10"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="7"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B2:F3"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>